<commit_message>
MTE CZ26011717: HS 9027 89 90 confirmed, lancets 9018 90 84 confirmed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011XkebLxGdjGSmsotkzP3mB
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_MTE_CZ26011717.xlsx
+++ b/output/HS_Code_Summary_MTE_CZ26011717.xlsx
@@ -105,6 +105,18 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -115,18 +127,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -609,7 +609,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>90278900</t>
+          <t>90278990</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -644,110 +644,106 @@
       <c r="I4" s="7" t="n">
         <v>13980</v>
       </c>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>KONTROLA KN</t>
-        </is>
-      </c>
+      <c r="J4" s="4" t="inlineStr"/>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>Kód dle klienta 90278900 (faktura 9027.89). Podpoložka KN 9027 89 00 v KN nemusí existovat (9027 89 je dále členěna) – ověřit 8místný kód v TARIC před podáním.</t>
+          <t>KN 9027 89 90 – potvrzeno (klient uvedl 90278900, faktura 9027.89; opraveno na platnou podpoložku KN).</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>38221900</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Testovací proužky do glukometrů FORA 6 (7650bal.); Testovací proužky do glukometrů FORA 6 Beta-ketony  (720bal.); Testovací proužky do glukometrů FORA Diamond (26250bal.)</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>ForaCare Suisse AG (CH)</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>TW</t>
         </is>
       </c>
-      <c r="E5" s="9" t="n">
+      <c r="E5" s="5" t="n">
         <v>34620</v>
       </c>
-      <c r="F5" s="8" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>bal.</t>
         </is>
       </c>
-      <c r="G5" s="10" t="n">
+      <c r="G5" s="6" t="n">
         <v>1821.415</v>
       </c>
-      <c r="H5" s="10" t="n">
+      <c r="H5" s="6" t="n">
         <v>2044.172</v>
       </c>
-      <c r="I5" s="11" t="n">
+      <c r="I5" s="7" t="n">
         <v>236859</v>
       </c>
-      <c r="J5" s="8" t="inlineStr"/>
-      <c r="K5" s="8" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr"/>
+      <c r="K5" s="4" t="inlineStr">
         <is>
           <t>Kód dle klienta i faktury (3822.19). Diagnostická činidla na podložce – in-vitro.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>85235110</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Elektronický teploměr (2 kusy)</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>ForaCare Suisse AG (CH)</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>?</t>
         </is>
       </c>
-      <c r="E6" s="5" t="n">
+      <c r="E6" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F6" s="8" t="inlineStr">
         <is>
           <t>ks</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="G6" s="10" t="inlineStr">
         <is>
           <t>neuvedeno</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="H6" s="10" t="inlineStr">
         <is>
           <t>neuvedeno</t>
         </is>
       </c>
-      <c r="I6" s="7" t="n">
+      <c r="I6" s="11" t="n">
         <v>70</v>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="J6" s="8" t="inlineStr">
         <is>
           <t>KONTROLA</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr">
+      <c r="K6" s="8" t="inlineStr">
         <is>
           <t>Kód dle klienta 85235110. Na faktuře jako „Temperature monitor fee (SEA)“ 2×35 USD; v packing listu není (bez hmotnosti a původu). Klient popisuje jako elektronický teploměr → zvážit 9025 19 00; ověřit zda jde o zboží nebo poplatek.</t>
         </is>
@@ -877,45 +873,45 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>38221900</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Testovací proužky do glukometrů FORA 6 (3750bal.); Testovací proužky do glukometrů FORA Diamond (8750bal.); Kontrolní roztok Level 2 (150bal.); Kontrolní roztok Level 3 (50bal.)</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>ForaCare Suisse AG (CH)</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>TW</t>
         </is>
       </c>
-      <c r="E4" s="9" t="n">
+      <c r="E4" s="5" t="n">
         <v>12700</v>
       </c>
-      <c r="F4" s="8" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>bal.</t>
         </is>
       </c>
-      <c r="G4" s="10" t="n">
+      <c r="G4" s="6" t="n">
         <v>665.255</v>
       </c>
-      <c r="H4" s="10" t="n">
+      <c r="H4" s="6" t="n">
         <v>747.498</v>
       </c>
-      <c r="I4" s="11" t="n">
+      <c r="I4" s="7" t="n">
         <v>85815</v>
       </c>
-      <c r="J4" s="8" t="inlineStr"/>
-      <c r="K4" s="8" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr"/>
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>Kód dle klienta i faktury (3822.19). Diagnostická činidla na podložce – in-vitro.</t>
         </is>
@@ -966,7 +962,7 @@
       </c>
       <c r="K5" s="16" t="inlineStr">
         <is>
-          <t>Klient i faktura uvádí jen 9018.90 (6 míst) → KN podpoložku dopočítáno pravidlem CCT/VPV KN: 9018 90 84 (ostatní nástroje a přístroje pro lékařství). NUTNO POTVRDIT. Původ CN (paleta S17, MADE IN CHINA).</t>
+          <t>Klient i faktura uvádí jen 9018.90 (6 míst) → KN podpoložka dopočítána pravidlem CCT/VPV KN: 9018 90 84 (ostatní nástroje a přístroje pro lékařství) – potvrzeno. Původ CN (paleta S17, MADE IN CHINA).</t>
         </is>
       </c>
     </row>
@@ -1192,7 +1188,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Pro dotčené kódy (3822 19 00, 9027 89, 9018 90 84, 8523 51 10) z TW/CN není znám antidumping – ověřit v TARIC při podání.</t>
+          <t>Pro dotčené kódy (3822 19 00, 9027 89 90, 9018 90 84, 8523 51 10) z TW/CN není znám antidumping – ověřit v TARIC při podání.</t>
         </is>
       </c>
     </row>
@@ -1229,7 +1225,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Nejistota: potvrdit, případně konzultovat customs.tariff@mauriceward.com.</t>
+          <t>Stav: 9018 90 84 potvrzeno.</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1269,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Pol. 10 (teploměry / „Temperature monitor fee“): hmotnost ani původ v dokladech NEJSOU.</t>
+          <t>Pol. 10 (teploměry / „Temperature monitor fee“): hmotnost ani původ v dokladech NEJSOU. OTEVŘENO – dotaz na L. Jirkovského: zboží vs. poplatek, HS kód, NW/GW, země původu.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
MTE CZ26011717: item 10 = temperature data loggers, HS 9025 19 00
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011XkebLxGdjGSmsotkzP3mB
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_MTE_CZ26011717.xlsx
+++ b/output/HS_Code_Summary_MTE_CZ26011717.xlsx
@@ -699,7 +699,7 @@
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>85235110</t>
+          <t>90251900</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
@@ -740,12 +740,12 @@
       </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
-          <t>KONTROLA</t>
+          <t>KONTROLA HMOTNOSTI</t>
         </is>
       </c>
       <c r="K6" s="8" t="inlineStr">
         <is>
-          <t>Kód dle klienta 85235110. Na faktuře jako „Temperature monitor fee (SEA)“ 2×35 USD; v packing listu není (bez hmotnosti a původu). Klient popisuje jako elektronický teploměr → zvážit 9025 19 00; ověřit zda jde o zboží nebo poplatek.</t>
+          <t>Dataloggery teploty v kontejneru (potvrzeno zákazníkem), dodavatel je přidává za úplatu → zboží v placené JSD. KN 9025 19 00 (elektronický teploměr) místo dříve používaného 85235110 – zákazník souhlasí. Hmotnost (NW/GW) a země původu zatím chybí – vyžádáno.</t>
         </is>
       </c>
     </row>
@@ -1188,7 +1188,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Pro dotčené kódy (3822 19 00, 9027 89 90, 9018 90 84, 8523 51 10) z TW/CN není znám antidumping – ověřit v TARIC při podání.</t>
+          <t>Pro dotčené kódy (3822 19 00, 9027 89 90, 9018 90 84, 9025 19 00) z TW/CN není znám antidumping – ověřit v TARIC při podání.</t>
         </is>
       </c>
     </row>
@@ -1269,7 +1269,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Pol. 10 (teploměry / „Temperature monitor fee“): hmotnost ani původ v dokladech NEJSOU. OTEVŘENO – dotaz na L. Jirkovského: zboží vs. poplatek, HS kód, NW/GW, země původu.</t>
+          <t>Pol. 10 (teploměry / „Temperature monitor fee“): hmotnost ani původ v dokladech NEJSOU. Zákazník potvrdil: dataloggery teploty, placené → JSD 1, HS 9025 19 00. OTEVŘENO: NW/GW a země původu.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
MTE CZ26011717: data logger weights (NW 30 g, GW 40 g) and origin TW
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011XkebLxGdjGSmsotkzP3mB
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_MTE_CZ26011717.xlsx
+++ b/output/HS_Code_Summary_MTE_CZ26011717.xlsx
@@ -44,17 +44,12 @@
       <i val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFE699"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -98,11 +93,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -117,40 +112,28 @@
     <xf numFmtId="4" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -697,82 +680,74 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>90251900</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Elektronický teploměr (2 kusy)</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>ForaCare Suisse AG (CH)</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
-      </c>
-      <c r="E6" s="9" t="n">
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>ks</t>
         </is>
       </c>
-      <c r="G6" s="10" t="inlineStr">
-        <is>
-          <t>neuvedeno</t>
-        </is>
-      </c>
-      <c r="H6" s="10" t="inlineStr">
-        <is>
-          <t>neuvedeno</t>
-        </is>
-      </c>
-      <c r="I6" s="11" t="n">
+      <c r="G6" s="6" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="I6" s="7" t="n">
         <v>70</v>
       </c>
-      <c r="J6" s="8" t="inlineStr">
-        <is>
-          <t>KONTROLA HMOTNOSTI</t>
-        </is>
-      </c>
-      <c r="K6" s="8" t="inlineStr">
-        <is>
-          <t>Dataloggery teploty v kontejneru (potvrzeno zákazníkem), dodavatel je přidává za úplatu → zboží v placené JSD. KN 9025 19 00 (elektronický teploměr) místo dříve používaného 85235110 – zákazník souhlasí. Hmotnost (NW/GW) a země původu zatím chybí – vyžádáno.</t>
+      <c r="J6" s="4" t="inlineStr"/>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>Dataloggery teploty v kontejneru (potvrzeno zákazníkem), placené → JSD 1. KN 9025 19 00 místo dříve používaného 85235110 – zákazník souhlasí. NW 30 g / GW 40 g, původ Taiwan – dle e-mailu L. Jirkovského 30.9.2026 (v PL nejsou).</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>CELKEM</t>
         </is>
       </c>
-      <c r="B7" s="12" t="inlineStr"/>
-      <c r="C7" s="12" t="inlineStr"/>
-      <c r="D7" s="12" t="inlineStr"/>
-      <c r="E7" s="13" t="n">
+      <c r="B7" s="8" t="inlineStr"/>
+      <c r="C7" s="8" t="inlineStr"/>
+      <c r="D7" s="8" t="inlineStr"/>
+      <c r="E7" s="9" t="n">
         <v>40622</v>
       </c>
-      <c r="F7" s="12" t="inlineStr"/>
-      <c r="G7" s="14" t="n">
-        <v>2706.415</v>
-      </c>
-      <c r="H7" s="14" t="n">
-        <v>3346.172</v>
-      </c>
-      <c r="I7" s="15" t="n">
+      <c r="F7" s="8" t="inlineStr"/>
+      <c r="G7" s="10" t="n">
+        <v>2706.445</v>
+      </c>
+      <c r="H7" s="10" t="n">
+        <v>3346.212</v>
+      </c>
+      <c r="I7" s="11" t="n">
         <v>250909</v>
       </c>
-      <c r="J7" s="12" t="inlineStr"/>
-      <c r="K7" s="12" t="inlineStr"/>
+      <c r="J7" s="8" t="inlineStr"/>
+      <c r="K7" s="8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -918,78 +893,78 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>90189084</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>Lancety FORA (10080 bal.) 50ks/bal.</t>
         </is>
       </c>
-      <c r="C5" s="16" t="inlineStr">
+      <c r="C5" s="12" t="inlineStr">
         <is>
           <t>ForaCare Suisse AG (CH)</t>
         </is>
       </c>
-      <c r="D5" s="16" t="inlineStr">
+      <c r="D5" s="12" t="inlineStr">
         <is>
           <t>CN</t>
         </is>
       </c>
-      <c r="E5" s="17" t="n">
+      <c r="E5" s="13" t="n">
         <v>10080</v>
       </c>
-      <c r="F5" s="16" t="inlineStr">
+      <c r="F5" s="12" t="inlineStr">
         <is>
           <t>bal.</t>
         </is>
       </c>
-      <c r="G5" s="18" t="n">
+      <c r="G5" s="14" t="n">
         <v>299.04</v>
       </c>
-      <c r="H5" s="18" t="n">
+      <c r="H5" s="14" t="n">
         <v>348.04</v>
       </c>
-      <c r="I5" s="19" t="n">
+      <c r="I5" s="15" t="n">
         <v>6048</v>
       </c>
-      <c r="J5" s="16" t="inlineStr">
+      <c r="J5" s="12" t="inlineStr">
         <is>
           <t>⚠ CCT/VPV KN</t>
         </is>
       </c>
-      <c r="K5" s="16" t="inlineStr">
+      <c r="K5" s="12" t="inlineStr">
         <is>
           <t>Klient i faktura uvádí jen 9018.90 (6 míst) → KN podpoložka dopočítána pravidlem CCT/VPV KN: 9018 90 84 (ostatní nástroje a přístroje pro lékařství) – potvrzeno. Původ CN (paleta S17, MADE IN CHINA).</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>CELKEM</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr"/>
-      <c r="C6" s="12" t="inlineStr"/>
-      <c r="D6" s="12" t="inlineStr"/>
-      <c r="E6" s="13" t="n">
+      <c r="B6" s="8" t="inlineStr"/>
+      <c r="C6" s="8" t="inlineStr"/>
+      <c r="D6" s="8" t="inlineStr"/>
+      <c r="E6" s="9" t="n">
         <v>22780</v>
       </c>
-      <c r="F6" s="12" t="inlineStr"/>
-      <c r="G6" s="14" t="n">
+      <c r="F6" s="8" t="inlineStr"/>
+      <c r="G6" s="10" t="n">
         <v>964.295</v>
       </c>
-      <c r="H6" s="14" t="n">
+      <c r="H6" s="10" t="n">
         <v>1095.538</v>
       </c>
-      <c r="I6" s="15" t="n">
+      <c r="I6" s="11" t="n">
         <v>91863</v>
       </c>
-      <c r="J6" s="12" t="inlineStr"/>
-      <c r="K6" s="12" t="inlineStr"/>
+      <c r="J6" s="8" t="inlineStr"/>
+      <c r="K6" s="8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1002,14 +977,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A43"/>
+  <dimension ref="A1:A46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="20">
+      <c r="A1" s="16">
         <f>== ZÁSILKA ===</f>
         <v/>
       </c>
@@ -1067,7 +1042,7 @@
       <c r="A9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="20">
+      <c r="A10" s="16">
         <f>== DVĚ JSD (instrukce zákazníka) ===</f>
         <v/>
       </c>
@@ -1104,7 +1079,7 @@
       <c r="A15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="20">
+      <c r="A16" s="16">
         <f>== INCOTERM ===</f>
         <v/>
       </c>
@@ -1127,7 +1102,7 @@
       <c r="A19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="20">
+      <c r="A20" s="16">
         <f>== PREFERENČNÍ PŮVOD / REX ===</f>
         <v/>
       </c>
@@ -1157,7 +1132,7 @@
       <c r="A24" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="20">
+      <c r="A25" s="16">
         <f>== CBAM ===</f>
         <v/>
       </c>
@@ -1180,7 +1155,7 @@
       <c r="A28" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="20">
+      <c r="A29" s="16">
         <f>== ANTIDUMPING ===</f>
         <v/>
       </c>
@@ -1196,80 +1171,96 @@
       <c r="A31" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="20">
+      <c r="A32" s="16">
+        <f>== MELT AND POUR ===</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Zásilka neobsahuje zboží ze železa/oceli (kap. 72/73) → pravidlo melt and pour se neuplatní.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="16">
         <f>== ⚠ CCT/VPV KN TARIFF RULE ===</f>
         <v/>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Lancety FORA (pol. 7): zdroj uvádí jen 9018.90 → KN 9018 90 84 odvozeno pravidlem CCT/VPV KN.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>CO TO JE? sterilní lanceta (jehlička) pro odběr kapilární krve. Z ČEHO? ocelový hrot v plastovém těle. K ČEMU? lékařský nástroj pro odběr krve (glukometrie).</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Třída XVIII, kap. 90 → čís. 9018 (nástroje pro lékařství) → 9018 90 (ostatní nástroje) → KN 9018 90 84 (ostatní). 9018 32 vyloučeno (pouze trubkové kovové jehly a jehly na šití); VPV 1 a 6.</t>
-        </is>
-      </c>
-    </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>Lancety FORA (pol. 7): zdroj uvádí jen 9018.90 → KN 9018 90 84 odvozeno pravidlem CCT/VPV KN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>CO TO JE? sterilní lanceta (jehlička) pro odběr kapilární krve. Z ČEHO? ocelový hrot v plastovém těle. K ČEMU? lékařský nástroj pro odběr krve (glukometrie).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Třída XVIII, kap. 90 → čís. 9018 (nástroje pro lékařství) → 9018 90 (ostatní nástroje) → KN 9018 90 84 (ostatní). 9018 32 vyloučeno (pouze trubkové kovové jehly a jehly na šití); VPV 1 a 6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>Stav: 9018 90 84 potvrzeno.</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="20">
+    <row r="40">
+      <c r="A40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="16">
         <f>== HMOTNOSTI ===</f>
         <v/>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Čistá hmotnost celkem 3 670,71 kg (PL). Hrubá 4 441,71 kg (PL paletový + HBL) = kartony 4 322,71 kg + palety 17 × 7 kg.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Rozpočet na HS kód: dle PL po produktech; paletová tára přiřazena po skupinách palet (S1–S6 monitor, S7–S16 proužky/roztoky, S17 lancety).</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Proužky FORA 6 a Diamond jsou částečně placené a částečně FOC → NW/GW rozděleno poměrem množství. Paleta S16 je smíšená (obě JSD).</t>
-        </is>
-      </c>
-    </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Kontrolní roztoky Level 2/3 v jedné krabici SDL1 (GW 3,63 kg) → GW rozděleno poměrem NW.</t>
+          <t>Čistá hmotnost celkem 3 670,71 kg (PL). Hrubá 4 441,71 kg (PL paletový + HBL) = kartony 4 322,71 kg + palety 17 × 7 kg.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Pol. 10 (teploměry / „Temperature monitor fee“): hmotnost ani původ v dokladech NEJSOU. Zákazník potvrdil: dataloggery teploty, placené → JSD 1, HS 9025 19 00. OTEVŘENO: NW/GW a země původu.</t>
+          <t>Rozpočet na HS kód: dle PL po produktech; paletová tára přiřazena po skupinách palet (S1–S6 monitor, S7–S16 proužky/roztoky, S17 lancety).</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Proužky FORA 6 a Diamond jsou částečně placené a částečně FOC → NW/GW rozděleno poměrem množství. Paleta S16 je smíšená (obě JSD).</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Kontrolní roztoky Level 2/3 v jedné krabici SDL1 (GW 3,63 kg) → GW rozděleno poměrem NW.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Pol. 10 (teploměry / „Temperature monitor fee“): hmotnost ani původ v dokladech NEJSOU. Zákazník potvrdil: dataloggery teploty, placené → JSD 1, HS 9025 19 00. NW 0,030 kg, GW 0,040 kg (celkem za 2 ks), původ TW – e-mail L. Jirkovského 30.9.2026. Nejsou v PL ani v HBL → celková GW obou JSD 4 441,75 kg vs. HBL 4 441,71 kg (+0,04 kg).</t>
         </is>
       </c>
     </row>

</xml_diff>